<commit_message>
Refine trade elasticities workflow outputs
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx
+++ b/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
@@ -463,7 +463,7 @@
         <v>27.6</v>
       </c>
       <c r="J2" s="2">
-        <v>46163.87687749697</v>
+        <v>46164.04494451366</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         <v>22.6</v>
       </c>
       <c r="J3" s="2">
-        <v>46163.87687811721</v>
+        <v>46164.04494599711</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         <v>74.8</v>
       </c>
       <c r="J4" s="2">
-        <v>46163.87688721895</v>
+        <v>46164.04495545782</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>81.2</v>
       </c>
       <c r="J5" s="2">
-        <v>46163.87688794706</v>
+        <v>46164.04495649236</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         <v>80.09999999999999</v>
       </c>
       <c r="J6" s="2">
-        <v>46163.87715495783</v>
+        <v>46164.04521096623</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>218.2</v>
       </c>
       <c r="J7" s="2">
-        <v>46163.87692318784</v>
+        <v>46164.04499186315</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         <v>257.5</v>
       </c>
       <c r="J8" s="2">
-        <v>46163.87695117849</v>
+        <v>46164.0450132938</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         <v>423.4</v>
       </c>
       <c r="J9" s="2">
-        <v>46163.87696824734</v>
+        <v>46164.04502917228</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>288.4</v>
       </c>
       <c r="J10" s="2">
-        <v>46163.87699306819</v>
+        <v>46164.04504758459</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>71.90000000000001</v>
       </c>
       <c r="J11" s="2">
-        <v>46163.87700694714</v>
+        <v>46164.04505974601</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
         <v>268.4</v>
       </c>
       <c r="J12" s="2">
-        <v>46163.87725839407</v>
+        <v>46164.04530607979</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1021,10 +1021,10 @@
         <v>1</v>
       </c>
       <c r="I13">
-        <v>380.7</v>
+        <v>341</v>
       </c>
       <c r="J13" s="2">
-        <v>46163.87727602477</v>
+        <v>46164.04532310629</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1072,10 +1072,10 @@
         <v>1</v>
       </c>
       <c r="I14">
-        <v>318.9</v>
+        <v>256.1</v>
       </c>
       <c r="J14" s="2">
-        <v>46163.87729250808</v>
+        <v>46164.04533763552</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1123,10 +1123,10 @@
         <v>1</v>
       </c>
       <c r="I15">
-        <v>111.1</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="J15" s="2">
-        <v>46163.8773010783</v>
+        <v>46164.04534581763</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1174,10 +1174,10 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="J16" s="2">
-        <v>46163.87702716432</v>
+        <v>46164.04508066745</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1225,10 +1225,10 @@
         <v>1</v>
       </c>
       <c r="I17">
-        <v>16.8</v>
+        <v>19.3</v>
       </c>
       <c r="J17" s="2">
-        <v>46163.8771557182</v>
+        <v>46164.04521449018</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1276,10 +1276,10 @@
         <v>1</v>
       </c>
       <c r="I18">
-        <v>28.8</v>
+        <v>26.9</v>
       </c>
       <c r="J18" s="2">
-        <v>46163.87723573948</v>
+        <v>46164.04528336697</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1327,10 +1327,10 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
       <c r="J19" s="2">
-        <v>46163.87724434903</v>
+        <v>46164.04529142848</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         <v>0.7</v>
       </c>
       <c r="J20" s="2">
-        <v>46163.87723473566</v>
+        <v>46164.04528190233</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>final_outputs_index.xlsx</t>
+          <t>literature_comparison_template.csv</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1407,36 +1407,36 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>control de entrega</t>
+          <t>cuadro comparativo para informe</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>indice de archivos finales generado por la seccion 13</t>
+          <t>plantilla para comparar elasticidades con literatura sugerida</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/literature_comparison_template.csv</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21">
-        <v>8.800000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="J21" s="2">
-        <v>46163.86794735471</v>
+        <v>46164.04528218386</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>se genera al correr esta seccion</t>
+          <t>disponible</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>section_14_reproducibility_check.xlsx</t>
+          <t>final_outputs_index.xlsx</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1463,31 +1463,31 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>control de reproducibilidad</t>
+          <t>control de entrega</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>checklist final de reproducibilidad generado por la seccion 14</t>
+          <t>indice de archivos finales generado por la seccion 13</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_14_reproducibility_check.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J22" s="2">
-        <v>46163.86833316211</v>
+        <v>46164.03617005008</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>se genera en la seccion 14</t>
+          <t>se genera al correr esta seccion</t>
         </is>
       </c>
     </row>
@@ -1499,46 +1499,244 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>section_14_reproducibility_check.xlsx</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>xlsx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>control de reproducibilidad</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>checklist final de reproducibilidad generado por la seccion 14</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_14_reproducibility_check.xlsx</t>
+        </is>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>9.1</v>
+      </c>
+      <c r="J23" s="2">
+        <v>46164.03617483603</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>se genera en la seccion 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>trazabilidad</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>session_info.txt</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>txt</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>control de reproducibilidad</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>informacion de sesion R generada por la seccion 14</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/session_info.txt</t>
         </is>
       </c>
-      <c r="H23" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23">
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24">
         <v>1.9</v>
       </c>
-      <c r="J23" s="2">
-        <v>46163.86838411585</v>
-      </c>
-      <c r="K23" t="inlineStr">
+      <c r="J24" s="2">
+        <v>46164.03617579181</v>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>se genera en la seccion 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>entrega</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>trade-elasticities-cointegration-report.pdf</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>entrega final</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>informe final en PDF</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.pdf</t>
+        </is>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>17.9</v>
+      </c>
+      <c r="J25" s="2">
+        <v>46157.6505310852</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>disponible</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>entrega</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>trade-elasticities-cointegration-report.docx</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>entrega final</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>informe final en Word</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.docx</t>
+        </is>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>pendiente: generar fuera del script</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>entrega</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>trade_elasticities_cointegration.R</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/scripts</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>entrega final</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>script R reproducible</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/scripts/trade_elasticities_cointegration.R</t>
+        </is>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>133.7</v>
+      </c>
+      <c r="J27" s="2">
+        <v>46164.04059739185</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>disponible</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1817,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1657,7 +1855,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>figura</t>
+          <t>entrega</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1666,28 +1864,28 @@
         </is>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tabla econometrica</t>
+          <t>entrega</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>disponible</t>
+          <t>pendiente: generar fuera del script</t>
         </is>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>trazabilidad</t>
+          <t>figura</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1696,22 +1894,22 @@
         </is>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>trazabilidad</t>
+          <t>tabla econometrica</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>se genera al correr esta seccion</t>
+          <t>disponible</t>
         </is>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1722,10 +1920,40 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>disponible</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>trazabilidad</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>se genera al correr esta seccion</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>trazabilidad</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>se genera en la seccion 14</t>
         </is>
       </c>
-      <c r="C7">
+      <c r="C9">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Draft trade elasticities report results
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx
+++ b/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
@@ -463,7 +463,7 @@
         <v>27.6</v>
       </c>
       <c r="J2" s="2">
-        <v>46164.04494451366</v>
+        <v>46164.80581280815</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         <v>22.6</v>
       </c>
       <c r="J3" s="2">
-        <v>46164.04494599711</v>
+        <v>46164.80581308842</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         <v>74.8</v>
       </c>
       <c r="J4" s="2">
-        <v>46164.04495545782</v>
+        <v>46164.80581610401</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>81.2</v>
       </c>
       <c r="J5" s="2">
-        <v>46164.04495649236</v>
+        <v>46164.80581645418</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         <v>80.09999999999999</v>
       </c>
       <c r="J6" s="2">
-        <v>46164.04521096623</v>
+        <v>46164.80590850881</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -715,10 +715,10 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>218.2</v>
+        <v>212.9</v>
       </c>
       <c r="J7" s="2">
-        <v>46164.04499186315</v>
+        <v>46164.80582509504</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>logs de exportaciones, PIB socios, ITCRM y commodities</t>
+          <t>logs de exportaciones, PIB socios y commodities</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -766,10 +766,10 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>257.5</v>
+        <v>224.2</v>
       </c>
       <c r="J8" s="2">
-        <v>46164.0450132938</v>
+        <v>46164.8058309164</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>423.4</v>
+        <v>426.7</v>
       </c>
       <c r="J9" s="2">
-        <v>46164.04502917228</v>
+        <v>46164.80583622403</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -868,10 +868,10 @@
         <v>1</v>
       </c>
       <c r="I10">
-        <v>288.4</v>
+        <v>284.6</v>
       </c>
       <c r="J10" s="2">
-        <v>46164.04504758459</v>
+        <v>46164.80584187122</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         <v>1</v>
       </c>
       <c r="I11">
-        <v>71.90000000000001</v>
+        <v>61.2</v>
       </c>
       <c r="J11" s="2">
-        <v>46164.04505974601</v>
+        <v>46164.80584542451</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -970,10 +970,10 @@
         <v>1</v>
       </c>
       <c r="I12">
-        <v>268.4</v>
+        <v>261.7</v>
       </c>
       <c r="J12" s="2">
-        <v>46164.04530607979</v>
+        <v>46164.80594485601</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1021,10 +1021,10 @@
         <v>1</v>
       </c>
       <c r="I13">
-        <v>341</v>
+        <v>338.3</v>
       </c>
       <c r="J13" s="2">
-        <v>46164.04532310629</v>
+        <v>46164.80595178812</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>section_12_fitted_vs_residuals.png</t>
+          <t>section_12_fitted_vs_residuals_exports.png</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1060,22 +1060,22 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>valores ajustados vs residuos</t>
+          <t>valores ajustados vs residuos de exportaciones</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures/section_12_fitted_vs_residuals.png</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures/section_12_fitted_vs_residuals_exports.png</t>
         </is>
       </c>
       <c r="H14" t="b">
         <v>1</v>
       </c>
       <c r="I14">
-        <v>256.1</v>
+        <v>98.5</v>
       </c>
       <c r="J14" s="2">
-        <v>46164.04533763552</v>
+        <v>46164.80595460731</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>section_12_ecm_adjustment_speed.png</t>
+          <t>section_12_fitted_vs_residuals_imports.png</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1106,27 +1106,27 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>figura principal o anexo</t>
+          <t>anexo econometrico</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>velocidad de ajuste ECM</t>
+          <t>valores ajustados vs residuos de importaciones</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures/section_12_ecm_adjustment_speed.png</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures/section_12_fitted_vs_residuals_imports.png</t>
         </is>
       </c>
       <c r="H15" t="b">
         <v>1</v>
       </c>
       <c r="I15">
-        <v>98.59999999999999</v>
+        <v>174.9</v>
       </c>
       <c r="J15" s="2">
-        <v>46164.04534581763</v>
+        <v>46164.80595974906</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1137,47 +1137,47 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tabla econometrica</t>
+          <t>figura</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>section_09_stationarity_results.xlsx</t>
+          <t>section_12_ecm_adjustment_speed.png</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>png</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>anexo econometrico</t>
+          <t>figura principal o anexo</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>pruebas ADF, PP, KPSS y orden de integracion</t>
+          <t>velocidad de ajuste ECM</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_09_stationarity_results.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/figures/section_12_ecm_adjustment_speed.png</t>
         </is>
       </c>
       <c r="H16" t="b">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>13.1</v>
+        <v>62.2</v>
       </c>
       <c r="J16" s="2">
-        <v>46164.04508066745</v>
+        <v>46164.80596366632</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>section_10_cointegration_results.xlsx</t>
+          <t>section_09_stationarity_results.xlsx</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1213,22 +1213,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Engle-Granger, Gregory-Hansen y residuos de cointegracion</t>
+          <t>pruebas ADF, PP, KPSS y orden de integracion</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_10_cointegration_results.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_09_stationarity_results.xlsx</t>
         </is>
       </c>
       <c r="H17" t="b">
         <v>1</v>
       </c>
       <c r="I17">
-        <v>19.3</v>
+        <v>13.1</v>
       </c>
       <c r="J17" s="2">
-        <v>46164.04521449018</v>
+        <v>46164.80585336244</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>section_11_econometric_models.xlsx</t>
+          <t>section_10_cointegration_results.xlsx</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1259,27 +1259,27 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>tabla principal y anexo</t>
+          <t>anexo econometrico</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>modelos ECM/diferencias, HAC, seleccion de rezagos y robustez</t>
+          <t>Engle-Granger, Gregory-Hansen y residuos de cointegracion</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_11_econometric_models.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_10_cointegration_results.xlsx</t>
         </is>
       </c>
       <c r="H18" t="b">
         <v>1</v>
       </c>
       <c r="I18">
-        <v>26.9</v>
+        <v>19.3</v>
       </c>
       <c r="J18" s="2">
-        <v>46164.04528336697</v>
+        <v>46164.80590885968</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>section_12_model_diagnostics.xlsx</t>
+          <t>section_11_econometric_models.xlsx</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1310,27 +1310,27 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>anexo econometrico</t>
+          <t>tabla principal y anexo</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>diagnosticos post-estimacion y lectura econometrica</t>
+          <t>modelos ECM/diferencias, HAC, seleccion de rezagos y robustez</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_12_model_diagnostics.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_11_econometric_models.xlsx</t>
         </is>
       </c>
       <c r="H19" t="b">
         <v>1</v>
       </c>
       <c r="I19">
-        <v>10.3</v>
+        <v>26.9</v>
       </c>
       <c r="J19" s="2">
-        <v>46164.04529142848</v>
+        <v>46164.80593668271</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1341,12 +1341,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>trazabilidad</t>
+          <t>tabla econometrica</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>pib_socios_traceability.csv</t>
+          <t>section_12_model_diagnostics.xlsx</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1356,32 +1356,32 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>anexo metodologico</t>
+          <t>anexo econometrico</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ponderadores originales y normalizados usados en PIBSOCIOS</t>
+          <t>diagnosticos post-estimacion y lectura econometrica</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/pib_socios_traceability.csv</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_12_model_diagnostics.xlsx</t>
         </is>
       </c>
       <c r="H20" t="b">
         <v>1</v>
       </c>
       <c r="I20">
-        <v>0.7</v>
+        <v>10.3</v>
       </c>
       <c r="J20" s="2">
-        <v>46164.04528190233</v>
+        <v>46164.80594031976</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>literature_comparison_template.csv</t>
+          <t>pib_socios_traceability.csv</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1412,27 +1412,27 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>cuadro comparativo para informe</t>
+          <t>anexo metodologico</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>plantilla para comparar elasticidades con literatura sugerida</t>
+          <t>ponderadores originales y normalizados usados en PIBSOCIOS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/literature_comparison_template.csv</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/pib_socios_traceability.csv</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="J21" s="2">
-        <v>46164.04528218386</v>
+        <v>46164.80593619278</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>final_outputs_index.xlsx</t>
+          <t>literature_comparison_template.csv</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1458,36 +1458,36 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>control de entrega</t>
+          <t>cuadro comparativo para informe</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>indice de archivos finales generado por la seccion 13</t>
+          <t>plantilla para comparar elasticidades con literatura sugerida</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/literature_comparison_template.csv</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22">
-        <v>9.199999999999999</v>
+        <v>1.4</v>
       </c>
       <c r="J22" s="2">
-        <v>46164.03617005008</v>
+        <v>46164.80593628643</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>se genera al correr esta seccion</t>
+          <t>disponible</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>section_14_reproducibility_check.xlsx</t>
+          <t>final_outputs_index.xlsx</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1514,31 +1514,31 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>control de reproducibilidad</t>
+          <t>control de entrega</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>checklist final de reproducibilidad generado por la seccion 14</t>
+          <t>indice de archivos finales generado por la seccion 13</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_14_reproducibility_check.xlsx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/final_outputs_index.xlsx</t>
         </is>
       </c>
       <c r="H23" t="b">
         <v>1</v>
       </c>
       <c r="I23">
-        <v>9.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J23" s="2">
-        <v>46164.03617483603</v>
+        <v>46164.80191181571</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>se genera en la seccion 14</t>
+          <t>se genera al correr esta seccion</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>session_info.txt</t>
+          <t>section_14_reproducibility_check.xlsx</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>txt</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1570,22 +1570,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>informacion de sesion R generada por la seccion 14</t>
+          <t>checklist final de reproducibilidad generado por la seccion 14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/session_info.txt</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/section_14_reproducibility_check.xlsx</t>
         </is>
       </c>
       <c r="H24" t="b">
         <v>1</v>
       </c>
       <c r="I24">
-        <v>1.9</v>
+        <v>9.1</v>
       </c>
       <c r="J24" s="2">
-        <v>46164.03617579181</v>
+        <v>46164.80191385114</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1596,51 +1596,51 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>entrega</t>
+          <t>trazabilidad</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>trade-elasticities-cointegration-report.pdf</t>
+          <t>session_info.txt</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>entrega final</t>
+          <t>control de reproducibilidad</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>informe final en PDF</t>
+          <t>informacion de sesion R generada por la seccion 14</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.pdf</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/outputs/session_info.txt</t>
         </is>
       </c>
       <c r="H25" t="b">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>17.9</v>
+        <v>1.9</v>
       </c>
       <c r="J25" s="2">
-        <v>46157.6505310852</v>
+        <v>46164.80191414166</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>disponible</t>
+          <t>se genera en la seccion 14</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>trade-elasticities-cointegration-report.docx</t>
+          <t>trade-elasticities-cointegration-report.pdf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1672,20 +1672,26 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>informe final en Word</t>
+          <t>informe final en PDF</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.docx</t>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.pdf</t>
         </is>
       </c>
       <c r="H26" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>2304.1</v>
+      </c>
+      <c r="J26" s="2">
+        <v>46164.79643431447</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>pendiente: generar fuera del script</t>
+          <t>disponible</t>
         </is>
       </c>
     </row>
@@ -1697,44 +1703,89 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>trade-elasticities-cointegration-report.docx</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>entrega final</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>informe final en Word</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/report/trade-elasticities-cointegration-report.docx</t>
+        </is>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>pendiente: generar fuera del script</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>entrega</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>trade_elasticities_cointegration.R</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/scripts</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>entrega final</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>script R reproducible</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>C:/Users/julla/GitHub/applied-time-series-econometrics/trade-elasticities-cointegration/scripts/trade_elasticities_cointegration.R</t>
         </is>
       </c>
-      <c r="H27" t="b">
-        <v>1</v>
-      </c>
-      <c r="I27">
-        <v>133.7</v>
-      </c>
-      <c r="J27" s="2">
-        <v>46164.04059739185</v>
-      </c>
-      <c r="K27" t="inlineStr">
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28">
+        <v>133.5</v>
+      </c>
+      <c r="J28" s="2">
+        <v>46164.7993114873</v>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
@@ -1894,7 +1945,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">

</xml_diff>